<commit_message>
Rerun: sectoral-synergy study (required grid decarbonisation) on the corrected model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVt5c2AiN5SahjfAqCCvTJ
</commit_message>
<xml_diff>
--- a/structural/feasibility_and_synergy/sectoral_synergy/data/sectoral_synergy.xlsx
+++ b/structural/feasibility_and_synergy/sectoral_synergy/data/sectoral_synergy.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="5">
   <si>
     <t>h2_start</t>
   </si>
@@ -35,16 +35,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -60,7 +52,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -68,30 +60,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -390,16 +364,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -410,11 +384,8 @@
       <c r="B2">
         <v>0.01</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
+      <c r="D2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -424,11 +395,8 @@
       <c r="B3">
         <v>0.02</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
+      <c r="D3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -438,11 +406,8 @@
       <c r="B4">
         <v>0.03</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
+      <c r="D4" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -522,11 +487,8 @@
       <c r="B10">
         <v>0.01</v>
       </c>
-      <c r="C10">
-        <v>0.2969</v>
-      </c>
-      <c r="D10">
-        <v>29.69</v>
+      <c r="D10" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -536,11 +498,8 @@
       <c r="B11">
         <v>0.02</v>
       </c>
-      <c r="C11">
-        <v>0.2031</v>
-      </c>
-      <c r="D11">
-        <v>20.31</v>
+      <c r="D11" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -550,11 +509,8 @@
       <c r="B12">
         <v>0.03</v>
       </c>
-      <c r="C12">
-        <v>0.1094</v>
-      </c>
-      <c r="D12">
-        <v>10.94</v>
+      <c r="D12" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -564,11 +520,8 @@
       <c r="B13">
         <v>0.04</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
+      <c r="D13" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -578,11 +531,8 @@
       <c r="B14">
         <v>0.05</v>
       </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
+      <c r="D14" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -634,11 +584,8 @@
       <c r="B18">
         <v>0.01</v>
       </c>
-      <c r="C18">
-        <v>0.6094000000000001</v>
-      </c>
-      <c r="D18">
-        <v>60.94</v>
+      <c r="D18" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -648,11 +595,8 @@
       <c r="B19">
         <v>0.02</v>
       </c>
-      <c r="C19">
-        <v>0.4922</v>
-      </c>
-      <c r="D19">
-        <v>49.22</v>
+      <c r="D19" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -662,11 +606,8 @@
       <c r="B20">
         <v>0.03</v>
       </c>
-      <c r="C20">
-        <v>0.375</v>
-      </c>
-      <c r="D20">
-        <v>37.5</v>
+      <c r="D20" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -676,11 +617,8 @@
       <c r="B21">
         <v>0.04</v>
       </c>
-      <c r="C21">
-        <v>0.2422</v>
-      </c>
-      <c r="D21">
-        <v>24.22</v>
+      <c r="D21" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -690,11 +628,8 @@
       <c r="B22">
         <v>0.05</v>
       </c>
-      <c r="C22">
-        <v>0.1016</v>
-      </c>
-      <c r="D22">
-        <v>10.16</v>
+      <c r="D22" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -704,11 +639,8 @@
       <c r="B23">
         <v>0.06</v>
       </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
+      <c r="D23" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -746,11 +678,8 @@
       <c r="B26">
         <v>0.01</v>
       </c>
-      <c r="C26">
-        <v>0.8828</v>
-      </c>
-      <c r="D26">
-        <v>88.28</v>
+      <c r="D26" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -760,11 +689,8 @@
       <c r="B27">
         <v>0.02</v>
       </c>
-      <c r="C27">
-        <v>0.7578</v>
-      </c>
-      <c r="D27">
-        <v>75.78</v>
+      <c r="D27" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -774,11 +700,8 @@
       <c r="B28">
         <v>0.03</v>
       </c>
-      <c r="C28">
-        <v>0.6172</v>
-      </c>
-      <c r="D28">
-        <v>61.72</v>
+      <c r="D28" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -788,11 +711,8 @@
       <c r="B29">
         <v>0.04</v>
       </c>
-      <c r="C29">
-        <v>0.4688</v>
-      </c>
-      <c r="D29">
-        <v>46.88</v>
+      <c r="D29" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -802,11 +722,8 @@
       <c r="B30">
         <v>0.05</v>
       </c>
-      <c r="C30">
-        <v>0.2969</v>
-      </c>
-      <c r="D30">
-        <v>29.69</v>
+      <c r="D30" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -816,11 +733,8 @@
       <c r="B31">
         <v>0.06</v>
       </c>
-      <c r="C31">
-        <v>0.1172</v>
-      </c>
-      <c r="D31">
-        <v>11.72</v>
+      <c r="D31" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -830,11 +744,8 @@
       <c r="B32">
         <v>0.07000000000000001</v>
       </c>
-      <c r="C32">
-        <v>0</v>
-      </c>
-      <c r="D32">
-        <v>0</v>
+      <c r="D32" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -869,11 +780,8 @@
       <c r="B35">
         <v>0.02</v>
       </c>
-      <c r="C35">
-        <v>0.9688</v>
-      </c>
-      <c r="D35">
-        <v>96.88</v>
+      <c r="D35" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -883,11 +791,8 @@
       <c r="B36">
         <v>0.03</v>
       </c>
-      <c r="C36">
-        <v>0.8203</v>
-      </c>
-      <c r="D36">
-        <v>82.03</v>
+      <c r="D36" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -897,11 +802,8 @@
       <c r="B37">
         <v>0.04</v>
       </c>
-      <c r="C37">
-        <v>0.6484</v>
-      </c>
-      <c r="D37">
-        <v>64.84</v>
+      <c r="D37" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -911,11 +813,8 @@
       <c r="B38">
         <v>0.05</v>
       </c>
-      <c r="C38">
-        <v>0.4609</v>
-      </c>
-      <c r="D38">
-        <v>46.09</v>
+      <c r="D38" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -925,11 +824,8 @@
       <c r="B39">
         <v>0.06</v>
       </c>
-      <c r="C39">
-        <v>0.2578</v>
-      </c>
-      <c r="D39">
-        <v>25.78</v>
+      <c r="D39" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -939,11 +835,8 @@
       <c r="B40">
         <v>0.07000000000000001</v>
       </c>
-      <c r="C40">
-        <v>0.0625</v>
-      </c>
-      <c r="D40">
-        <v>6.25</v>
+      <c r="D40" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -953,11 +846,8 @@
       <c r="B41">
         <v>0.08</v>
       </c>
-      <c r="C41">
-        <v>0</v>
-      </c>
-      <c r="D41">
-        <v>0</v>
+      <c r="D41" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -989,11 +879,8 @@
       <c r="B44">
         <v>0.03</v>
       </c>
-      <c r="C44">
-        <v>0.9530999999999999</v>
-      </c>
-      <c r="D44">
-        <v>95.31</v>
+      <c r="D44" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -1003,11 +890,8 @@
       <c r="B45">
         <v>0.04</v>
       </c>
-      <c r="C45">
-        <v>0.7734</v>
-      </c>
-      <c r="D45">
-        <v>77.34</v>
+      <c r="D45" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -1017,11 +901,8 @@
       <c r="B46">
         <v>0.05</v>
       </c>
-      <c r="C46">
-        <v>0.5703</v>
-      </c>
-      <c r="D46">
-        <v>57.03</v>
+      <c r="D46" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -1031,11 +912,8 @@
       <c r="B47">
         <v>0.06</v>
       </c>
-      <c r="C47">
-        <v>0.3594</v>
-      </c>
-      <c r="D47">
-        <v>35.94</v>
+      <c r="D47" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -1045,11 +923,8 @@
       <c r="B48">
         <v>0.07000000000000001</v>
       </c>
-      <c r="C48">
-        <v>0.1484</v>
-      </c>
-      <c r="D48">
-        <v>14.84</v>
+      <c r="D48" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -1059,11 +934,8 @@
       <c r="B49">
         <v>0.08</v>
       </c>
-      <c r="C49">
-        <v>0</v>
-      </c>
-      <c r="D49">
-        <v>0</v>
+      <c r="D49" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rerun: sectoral synergy after the theta_grid = 1 fix
Required grid-emission offset now rises smoothly with H2 delay and falls
with scrap growth; much larger than in the paper (e.g. H2 2033 / scrap 4 %:
37 % vs 0 %). With H2 from 2036 and scrap growth <= 2 %, no grid
decarbonisation is enough.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVt5c2AiN5SahjfAqCCvTJ
</commit_message>
<xml_diff>
--- a/structural/feasibility_and_synergy/sectoral_synergy/data/sectoral_synergy.xlsx
+++ b/structural/feasibility_and_synergy/sectoral_synergy/data/sectoral_synergy.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="5">
   <si>
     <t>h2_start</t>
   </si>
@@ -384,8 +384,11 @@
       <c r="B2">
         <v>0.01</v>
       </c>
-      <c r="D2" t="s">
-        <v>4</v>
+      <c r="C2">
+        <v>0.3984</v>
+      </c>
+      <c r="D2">
+        <v>39.84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -395,8 +398,11 @@
       <c r="B3">
         <v>0.02</v>
       </c>
-      <c r="D3" t="s">
-        <v>4</v>
+      <c r="C3">
+        <v>0.2656</v>
+      </c>
+      <c r="D3">
+        <v>26.56</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -406,8 +412,11 @@
       <c r="B4">
         <v>0.03</v>
       </c>
-      <c r="D4" t="s">
-        <v>4</v>
+      <c r="C4">
+        <v>0.1016</v>
+      </c>
+      <c r="D4">
+        <v>10.16</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -487,8 +496,11 @@
       <c r="B10">
         <v>0.01</v>
       </c>
-      <c r="D10" t="s">
-        <v>4</v>
+      <c r="C10">
+        <v>0.8516</v>
+      </c>
+      <c r="D10">
+        <v>85.16</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -498,8 +510,11 @@
       <c r="B11">
         <v>0.02</v>
       </c>
-      <c r="D11" t="s">
-        <v>4</v>
+      <c r="C11">
+        <v>0.7109</v>
+      </c>
+      <c r="D11">
+        <v>71.09</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -509,8 +524,11 @@
       <c r="B12">
         <v>0.03</v>
       </c>
-      <c r="D12" t="s">
-        <v>4</v>
+      <c r="C12">
+        <v>0.5547</v>
+      </c>
+      <c r="D12">
+        <v>55.47</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -520,8 +538,11 @@
       <c r="B13">
         <v>0.04</v>
       </c>
-      <c r="D13" t="s">
-        <v>4</v>
+      <c r="C13">
+        <v>0.3672</v>
+      </c>
+      <c r="D13">
+        <v>36.72</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -531,8 +552,11 @@
       <c r="B14">
         <v>0.05</v>
       </c>
-      <c r="D14" t="s">
-        <v>4</v>
+      <c r="C14">
+        <v>0.1562</v>
+      </c>
+      <c r="D14">
+        <v>15.62</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -606,8 +630,11 @@
       <c r="B20">
         <v>0.03</v>
       </c>
-      <c r="D20" t="s">
-        <v>4</v>
+      <c r="C20">
+        <v>0.9530999999999999</v>
+      </c>
+      <c r="D20">
+        <v>95.31</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -617,8 +644,11 @@
       <c r="B21">
         <v>0.04</v>
       </c>
-      <c r="D21" t="s">
-        <v>4</v>
+      <c r="C21">
+        <v>0.7578</v>
+      </c>
+      <c r="D21">
+        <v>75.78</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -628,8 +658,11 @@
       <c r="B22">
         <v>0.05</v>
       </c>
-      <c r="D22" t="s">
-        <v>4</v>
+      <c r="C22">
+        <v>0.5312</v>
+      </c>
+      <c r="D22">
+        <v>53.12</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -639,8 +672,11 @@
       <c r="B23">
         <v>0.06</v>
       </c>
-      <c r="D23" t="s">
-        <v>4</v>
+      <c r="C23">
+        <v>0.2812</v>
+      </c>
+      <c r="D23">
+        <v>28.12</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -722,8 +758,11 @@
       <c r="B30">
         <v>0.05</v>
       </c>
-      <c r="D30" t="s">
-        <v>4</v>
+      <c r="C30">
+        <v>0.8438</v>
+      </c>
+      <c r="D30">
+        <v>84.38</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -733,8 +772,11 @@
       <c r="B31">
         <v>0.06</v>
       </c>
-      <c r="D31" t="s">
-        <v>4</v>
+      <c r="C31">
+        <v>0.5703</v>
+      </c>
+      <c r="D31">
+        <v>57.03</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -744,8 +786,11 @@
       <c r="B32">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D32" t="s">
-        <v>4</v>
+      <c r="C32">
+        <v>0.2656</v>
+      </c>
+      <c r="D32">
+        <v>26.56</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -824,8 +869,11 @@
       <c r="B39">
         <v>0.06</v>
       </c>
-      <c r="D39" t="s">
-        <v>4</v>
+      <c r="C39">
+        <v>0.7969000000000001</v>
+      </c>
+      <c r="D39">
+        <v>79.69</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -835,8 +883,11 @@
       <c r="B40">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D40" t="s">
-        <v>4</v>
+      <c r="C40">
+        <v>0.4688</v>
+      </c>
+      <c r="D40">
+        <v>46.88</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -846,8 +897,11 @@
       <c r="B41">
         <v>0.08</v>
       </c>
-      <c r="D41" t="s">
-        <v>4</v>
+      <c r="C41">
+        <v>0.0859</v>
+      </c>
+      <c r="D41">
+        <v>8.59</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -912,8 +966,11 @@
       <c r="B47">
         <v>0.06</v>
       </c>
-      <c r="D47" t="s">
-        <v>4</v>
+      <c r="C47">
+        <v>0.9530999999999999</v>
+      </c>
+      <c r="D47">
+        <v>95.31</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -923,8 +980,11 @@
       <c r="B48">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D48" t="s">
-        <v>4</v>
+      <c r="C48">
+        <v>0.6016</v>
+      </c>
+      <c r="D48">
+        <v>60.16</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -934,8 +994,11 @@
       <c r="B49">
         <v>0.08</v>
       </c>
-      <c r="D49" t="s">
-        <v>4</v>
+      <c r="C49">
+        <v>0.1953</v>
+      </c>
+      <c r="D49">
+        <v>19.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rerun with re-anchored bounds: feasibility drivers, H2 delay, fuel availability, synergy
Feasibility drivers (27,648 cells): 0.3 / 6.7 / 31.2 % feasible at targets
1.6 / 1.8 / 2.0 (old bounds 13 / 30 / 46 %; paper 27.6 / 41.5 / 54.0 %).
Sobol at 1.8: H2 start 0.65, scrap 0.45, H2 ramp 0.42, grid 0.30, coking coal
0.29, CCS 0.24, build budget 0.23, legacy 0.16, NG 0.10. At 1.8 a 0.25 CCS
ceiling triples feasibility against no CCS (12 % vs 4 %).

H2 delay (Fig. 3): 1.6 infeasible everywhere; 1.8 feasible only with H2 from
2030 at mid/high ramp (491 / 488 $/t); 2.0 feasible everywhere (468-472).
Fuel availability: only abundant coal + abundant NG with H2 from 2030.
Synergy: grid offsets of 80 % or more needed at low scrap; see data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVt5c2AiN5SahjfAqCCvTJ
</commit_message>
<xml_diff>
--- a/structural/feasibility_and_synergy/sectoral_synergy/data/sectoral_synergy.xlsx
+++ b/structural/feasibility_and_synergy/sectoral_synergy/data/sectoral_synergy.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="5">
   <si>
     <t>h2_start</t>
   </si>
@@ -384,11 +384,8 @@
       <c r="B2">
         <v>0.01</v>
       </c>
-      <c r="C2">
-        <v>0.3984</v>
-      </c>
-      <c r="D2">
-        <v>39.84</v>
+      <c r="D2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -398,11 +395,8 @@
       <c r="B3">
         <v>0.02</v>
       </c>
-      <c r="C3">
-        <v>0.2656</v>
-      </c>
-      <c r="D3">
-        <v>26.56</v>
+      <c r="D3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -413,10 +407,10 @@
         <v>0.03</v>
       </c>
       <c r="C4">
-        <v>0.1016</v>
+        <v>0.8359</v>
       </c>
       <c r="D4">
-        <v>10.16</v>
+        <v>83.59</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -427,10 +421,10 @@
         <v>0.04</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>0.625</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -441,10 +435,10 @@
         <v>0.05</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>0.3906</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -455,10 +449,10 @@
         <v>0.06</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>0.1172</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>11.72</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -496,11 +490,8 @@
       <c r="B10">
         <v>0.01</v>
       </c>
-      <c r="C10">
-        <v>0.8516</v>
-      </c>
-      <c r="D10">
-        <v>85.16</v>
+      <c r="D10" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -510,11 +501,8 @@
       <c r="B11">
         <v>0.02</v>
       </c>
-      <c r="C11">
-        <v>0.7109</v>
-      </c>
-      <c r="D11">
-        <v>71.09</v>
+      <c r="D11" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -524,11 +512,8 @@
       <c r="B12">
         <v>0.03</v>
       </c>
-      <c r="C12">
-        <v>0.5547</v>
-      </c>
-      <c r="D12">
-        <v>55.47</v>
+      <c r="D12" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -539,10 +524,10 @@
         <v>0.04</v>
       </c>
       <c r="C13">
-        <v>0.3672</v>
+        <v>0.9141</v>
       </c>
       <c r="D13">
-        <v>36.72</v>
+        <v>91.41</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -553,10 +538,10 @@
         <v>0.05</v>
       </c>
       <c r="C14">
-        <v>0.1562</v>
+        <v>0.6641</v>
       </c>
       <c r="D14">
-        <v>15.62</v>
+        <v>66.41</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -567,10 +552,10 @@
         <v>0.06</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>0.3906</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -581,10 +566,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>0.0781</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>7.81</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -630,11 +615,8 @@
       <c r="B20">
         <v>0.03</v>
       </c>
-      <c r="C20">
-        <v>0.9530999999999999</v>
-      </c>
-      <c r="D20">
-        <v>95.31</v>
+      <c r="D20" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -644,11 +626,8 @@
       <c r="B21">
         <v>0.04</v>
       </c>
-      <c r="C21">
-        <v>0.7578</v>
-      </c>
-      <c r="D21">
-        <v>75.78</v>
+      <c r="D21" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -659,10 +638,10 @@
         <v>0.05</v>
       </c>
       <c r="C22">
-        <v>0.5312</v>
+        <v>0.8984</v>
       </c>
       <c r="D22">
-        <v>53.12</v>
+        <v>89.84</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -673,10 +652,10 @@
         <v>0.06</v>
       </c>
       <c r="C23">
-        <v>0.2812</v>
+        <v>0.6094000000000001</v>
       </c>
       <c r="D23">
-        <v>28.12</v>
+        <v>60.94</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -687,10 +666,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>0.2969</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>29.69</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -758,11 +737,8 @@
       <c r="B30">
         <v>0.05</v>
       </c>
-      <c r="C30">
-        <v>0.8438</v>
-      </c>
-      <c r="D30">
-        <v>84.38</v>
+      <c r="D30" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -773,10 +749,10 @@
         <v>0.06</v>
       </c>
       <c r="C31">
-        <v>0.5703</v>
+        <v>0.7891</v>
       </c>
       <c r="D31">
-        <v>57.03</v>
+        <v>78.91</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -787,10 +763,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C32">
-        <v>0.2656</v>
+        <v>0.4531</v>
       </c>
       <c r="D32">
-        <v>26.56</v>
+        <v>45.31</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -801,10 +777,10 @@
         <v>0.08</v>
       </c>
       <c r="C33">
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -870,10 +846,10 @@
         <v>0.06</v>
       </c>
       <c r="C39">
-        <v>0.7969000000000001</v>
+        <v>0.9141</v>
       </c>
       <c r="D39">
-        <v>79.69</v>
+        <v>91.41</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -884,10 +860,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C40">
-        <v>0.4688</v>
+        <v>0.5703</v>
       </c>
       <c r="D40">
-        <v>46.88</v>
+        <v>57.03</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -898,10 +874,10 @@
         <v>0.08</v>
       </c>
       <c r="C41">
-        <v>0.0859</v>
+        <v>0.1641</v>
       </c>
       <c r="D41">
-        <v>8.59</v>
+        <v>16.41</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -967,10 +943,10 @@
         <v>0.06</v>
       </c>
       <c r="C47">
-        <v>0.9530999999999999</v>
+        <v>0.9922</v>
       </c>
       <c r="D47">
-        <v>95.31</v>
+        <v>99.22</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -981,10 +957,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C48">
-        <v>0.6016</v>
+        <v>0.6328</v>
       </c>
       <c r="D48">
-        <v>60.16</v>
+        <v>63.28</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -995,10 +971,10 @@
         <v>0.08</v>
       </c>
       <c r="C49">
-        <v>0.1953</v>
+        <v>0.2188</v>
       </c>
       <c r="D49">
-        <v>19.53</v>
+        <v>21.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>